<commit_message>
adjust magic extract ocr
</commit_message>
<xml_diff>
--- a/MagicCollection.xlsx
+++ b/MagicCollection.xlsx
@@ -338,7 +338,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2004"/>
+  <dimension ref="A1:Y2014"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="26.75" customWidth="1" style="9" min="1" max="1"/>
@@ -72582,70 +72582,574 @@
       </c>
     </row>
     <row r="1261">
-      <c r="G1261" s="7" t="n"/>
+      <c r="A1261" s="5" t="inlineStr">
+        <is>
+          <t>Gyre Engineer / Engenheiro da Espiral</t>
+        </is>
+      </c>
+      <c r="B1261" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Vedalken Wizard / Criatura — Vedalkeano Mago</t>
+        </is>
+      </c>
+      <c r="C1261" s="5" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D1261" s="5" t="inlineStr">
+        <is>
+          <t>{T}: Add {G}{U}. / {T}: Adicione {G}{U}.</t>
+        </is>
+      </c>
+      <c r="E1261" s="5" t="inlineStr">
+        <is>
+          <t>{1}{G}{U}</t>
+        </is>
+      </c>
+      <c r="F1261" s="5" t="inlineStr">
+        <is>
+          <t>Verde, Azul</t>
+        </is>
+      </c>
+      <c r="G1261" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1261" s="5" t="inlineStr">
+        <is>
+          <t>Ravnica Allegiance (RNA)</t>
+        </is>
+      </c>
+      <c r="I1261" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1261" s="5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K1261" s="8" t="n">
+        <v>46023</v>
+      </c>
+      <c r="L1261" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="M1261" s="7">
         <f>L1261*G1261</f>
         <v/>
       </c>
     </row>
     <row r="1262">
-      <c r="G1262" s="7" t="n"/>
+      <c r="A1262" s="5" t="inlineStr">
+        <is>
+          <t>Reknit / Retramar</t>
+        </is>
+      </c>
+      <c r="B1262" s="5" t="inlineStr">
+        <is>
+          <t>Instant / Mágica Instantânea</t>
+        </is>
+      </c>
+      <c r="C1262" s="5" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D1262" s="5" t="inlineStr">
+        <is>
+          <t>Regenerate target permanent. / Regenere a permanente alvo.</t>
+        </is>
+      </c>
+      <c r="E1262" s="5" t="inlineStr">
+        <is>
+          <t>{1}{G/W}</t>
+        </is>
+      </c>
+      <c r="F1262" s="5" t="inlineStr">
+        <is>
+          <t>Verde, Branco</t>
+        </is>
+      </c>
+      <c r="G1262" s="7" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H1262" s="5" t="inlineStr">
+        <is>
+          <t>Shadowmoor (SHM)</t>
+        </is>
+      </c>
+      <c r="I1262" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1262" s="5" t="n">
+        <v>2008</v>
+      </c>
+      <c r="L1262" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1262" s="7">
         <f>L1262*G1262</f>
         <v/>
       </c>
     </row>
     <row r="1263">
-      <c r="G1263" s="7" t="n"/>
+      <c r="A1263" s="5" t="inlineStr">
+        <is>
+          <t>Valeron Outlander / Forasteiro de Valeron</t>
+        </is>
+      </c>
+      <c r="B1263" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Human Scout / Criatura — Humano Batedor</t>
+        </is>
+      </c>
+      <c r="C1263" s="5" t="inlineStr">
+        <is>
+          <t>Common / Comum</t>
+        </is>
+      </c>
+      <c r="D1263" s="5" t="inlineStr">
+        <is>
+          <t>Protection from black / Proteção contra o preto</t>
+        </is>
+      </c>
+      <c r="E1263" s="5" t="inlineStr">
+        <is>
+          <t>{G}{W}</t>
+        </is>
+      </c>
+      <c r="F1263" s="5" t="inlineStr">
+        <is>
+          <t>Verde, Branco</t>
+        </is>
+      </c>
+      <c r="G1263" s="7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H1263" s="5" t="inlineStr">
+        <is>
+          <t>Conflux (CON)</t>
+        </is>
+      </c>
+      <c r="I1263" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1263" s="5" t="n">
+        <v>2009</v>
+      </c>
+      <c r="K1263" s="8" t="n">
+        <v>46055</v>
+      </c>
+      <c r="L1263" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="M1263" s="7">
         <f>L1263*G1263</f>
         <v/>
       </c>
     </row>
     <row r="1264">
-      <c r="G1264" s="7" t="n"/>
+      <c r="A1264" s="5" t="inlineStr">
+        <is>
+          <t>Sundering Growth / Crescimento Despedaçador</t>
+        </is>
+      </c>
+      <c r="B1264" s="5" t="inlineStr">
+        <is>
+          <t>Instant / Mágica Instantânea</t>
+        </is>
+      </c>
+      <c r="C1264" s="5" t="inlineStr">
+        <is>
+          <t>Common / Comum</t>
+        </is>
+      </c>
+      <c r="D1264" s="5" t="inlineStr">
+        <is>
+          <t>Destroy target artifact or enchantment, then populate. (Create a token that's a copy of a creature token you control.) / Destrua o artefato ou encantamento alvo e depois povoe. (Coloque no campo de batalha uma ficha que seja uma cópia de uma ficha de criatura que você controla.)</t>
+        </is>
+      </c>
+      <c r="E1264" s="5" t="inlineStr">
+        <is>
+          <t>{G/W}{G/W}</t>
+        </is>
+      </c>
+      <c r="F1264" s="5" t="inlineStr">
+        <is>
+          <t>Verde, Branco</t>
+        </is>
+      </c>
+      <c r="G1264" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H1264" s="5" t="inlineStr">
+        <is>
+          <t>Return to Ravnica (RTR)</t>
+        </is>
+      </c>
+      <c r="I1264" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1264" s="5" t="n">
+        <v>2012</v>
+      </c>
+      <c r="L1264" s="5" t="n">
+        <v>4</v>
+      </c>
       <c r="M1264" s="7">
         <f>L1264*G1264</f>
         <v/>
       </c>
     </row>
     <row r="1265">
-      <c r="G1265" s="7" t="n"/>
+      <c r="A1265" s="5" t="inlineStr">
+        <is>
+          <t>Architects of Will / Arquitetos do Arbítrio</t>
+        </is>
+      </c>
+      <c r="B1265" s="5" t="inlineStr">
+        <is>
+          <t>Artifact Creature — Human Wizard / Criatura Artefato — Humano Mago</t>
+        </is>
+      </c>
+      <c r="C1265" s="5" t="inlineStr">
+        <is>
+          <t>Common / Comum</t>
+        </is>
+      </c>
+      <c r="D1265" s="5" t="inlineStr">
+        <is>
+          <t>When this creature enters, look at the top three cards of target player's library, then put them back in any order. Cycling {U/B} ({U/B}, Discard this card: Draw a card.) / Quando Arquitetos do Arbítrio entrar em jogo, olhe os três cards do topo do grimório do jogador alvo, depois coloque-os de volta em qualquer ordem. Reciclar {U/B} ({U/B}, Descarte este card: Compre um card.)</t>
+        </is>
+      </c>
+      <c r="E1265" s="5" t="inlineStr">
+        <is>
+          <t>{2}{U}{B}</t>
+        </is>
+      </c>
+      <c r="F1265" s="5" t="inlineStr">
+        <is>
+          <t>Preto, Azul</t>
+        </is>
+      </c>
+      <c r="G1265" s="7" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="H1265" s="5" t="inlineStr">
+        <is>
+          <t>Alara Reborn (ARB)</t>
+        </is>
+      </c>
+      <c r="I1265" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1265" s="5" t="n">
+        <v>2009</v>
+      </c>
+      <c r="K1265" s="8" t="n">
+        <v>46084</v>
+      </c>
+      <c r="L1265" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1265" s="7">
         <f>L1265*G1265</f>
         <v/>
       </c>
     </row>
     <row r="1266">
-      <c r="G1266" s="7" t="n"/>
+      <c r="A1266" s="5" t="inlineStr">
+        <is>
+          <t>Fathom Feeder / Alimentador das Profundezas</t>
+        </is>
+      </c>
+      <c r="B1266" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Eldrazi Drone / Criatura — Eldrazi Zangão</t>
+        </is>
+      </c>
+      <c r="C1266" s="5" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D1266" s="5" t="inlineStr">
+        <is>
+          <t>Devoid (This card has no color.) Deathtouch Ingest (Whenever this creature deals combat damage to a player, that player exiles the top card of their library.) {3}{U}{B}: Draw a card. Each opponent exiles the top card of their library. / Desprovido (Este card não tem cor.)Toque mortíferoIngerir (Toda vez que esta criatura causa dano de combate a um jogador, ele exila o card do topo do próprio grimório.){3}{U}{B}: Compre um card. Cada oponente exila o card do topo do próprio grimório.</t>
+        </is>
+      </c>
+      <c r="E1266" s="5" t="inlineStr">
+        <is>
+          <t>{U}{B}</t>
+        </is>
+      </c>
+      <c r="F1266" s="5" t="inlineStr">
+        <is>
+          <t>Preto, Azul</t>
+        </is>
+      </c>
+      <c r="G1266" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H1266" s="5" t="inlineStr">
+        <is>
+          <t>Battle for Zendikar (BFZ)</t>
+        </is>
+      </c>
+      <c r="I1266" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1266" s="5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="K1266" s="8" t="n">
+        <v>46023</v>
+      </c>
+      <c r="L1266" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1266" s="7">
         <f>L1266*G1266</f>
         <v/>
       </c>
     </row>
     <row r="1267">
-      <c r="G1267" s="7" t="n"/>
+      <c r="A1267" s="5" t="inlineStr">
+        <is>
+          <t>Inkfathom Infiltrator / Infiltrado Braçatinta</t>
+        </is>
+      </c>
+      <c r="B1267" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Merfolk Rogue / Criatura — Tritão Ladino</t>
+        </is>
+      </c>
+      <c r="C1267" s="5" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D1267" s="5" t="inlineStr">
+        <is>
+          <t>This creature can't block and can't be blocked. / Infiltrado Braçatinta não pode bloquear e não pode ser bloqueado.</t>
+        </is>
+      </c>
+      <c r="E1267" s="5" t="inlineStr">
+        <is>
+          <t>{U/B}{U/B}</t>
+        </is>
+      </c>
+      <c r="F1267" s="5" t="inlineStr">
+        <is>
+          <t>Preto, Azul</t>
+        </is>
+      </c>
+      <c r="G1267" s="7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H1267" s="5" t="inlineStr">
+        <is>
+          <t>Shadowmoor (SHM)</t>
+        </is>
+      </c>
+      <c r="I1267" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1267" s="5" t="n">
+        <v>2008</v>
+      </c>
+      <c r="K1267" s="8" t="n">
+        <v>46024</v>
+      </c>
+      <c r="L1267" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1267" s="7">
         <f>L1267*G1267</f>
         <v/>
       </c>
     </row>
     <row r="1268">
-      <c r="G1268" s="7" t="n"/>
+      <c r="A1268" s="5" t="inlineStr">
+        <is>
+          <t>Gruul Spellbreaker / Quebra-mágicas Gruul</t>
+        </is>
+      </c>
+      <c r="B1268" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Ogre Warrior / Criatura — Ogro Guerreiro</t>
+        </is>
+      </c>
+      <c r="C1268" s="5" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D1268" s="5" t="inlineStr">
+        <is>
+          <t>Riot (This creature enters with your choice of a +1/+1 counter or haste.) Trample During your turn, you and this creature have hexproof. / Tumulto (Esta criatura entra no campo de batalha com um marcador +1/+1 ou ímpeto, à sua escolha.) Atropelar Enquanto for o seu turno, você e Quebra-mágicas Gruul têm resistência a magia.</t>
+        </is>
+      </c>
+      <c r="E1268" s="5" t="inlineStr">
+        <is>
+          <t>{1}{R}{G}</t>
+        </is>
+      </c>
+      <c r="F1268" s="5" t="inlineStr">
+        <is>
+          <t>Verde, Vermelho</t>
+        </is>
+      </c>
+      <c r="G1268" s="7" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="H1268" s="5" t="inlineStr">
+        <is>
+          <t>Ravnica Allegiance (RNA)</t>
+        </is>
+      </c>
+      <c r="I1268" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1268" s="5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="K1268" s="8" t="n">
+        <v>46084</v>
+      </c>
+      <c r="L1268" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1268" s="7">
         <f>L1268*G1268</f>
         <v/>
       </c>
     </row>
     <row r="1269">
-      <c r="G1269" s="7" t="n"/>
+      <c r="A1269" s="5" t="inlineStr">
+        <is>
+          <t>Judge's Familiar / Familiar do Juiz</t>
+        </is>
+      </c>
+      <c r="B1269" s="5" t="inlineStr">
+        <is>
+          <t>Creature — Bird / Criatura — Ave</t>
+        </is>
+      </c>
+      <c r="C1269" s="5" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D1269" s="5" t="inlineStr">
+        <is>
+          <t>Flying Sacrifice this creature: Counter target instant or sorcery spell unless its controller pays {1}. / Voar Sacrifique Familiar do Juiz: Anule a mágica instantânea ou feitiço alvo a menos que seu controlador pague {1}.</t>
+        </is>
+      </c>
+      <c r="E1269" s="5" t="inlineStr">
+        <is>
+          <t>{W/U}</t>
+        </is>
+      </c>
+      <c r="F1269" s="5" t="inlineStr">
+        <is>
+          <t>Azul, Branco</t>
+        </is>
+      </c>
+      <c r="G1269" s="7" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="H1269" s="5" t="inlineStr">
+        <is>
+          <t>Return to Ravnica (RTR)</t>
+        </is>
+      </c>
+      <c r="I1269" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1269" s="5" t="n">
+        <v>2012</v>
+      </c>
+      <c r="K1269" s="8" t="n">
+        <v>46023</v>
+      </c>
+      <c r="L1269" s="5" t="n">
+        <v>2</v>
+      </c>
       <c r="M1269" s="7">
         <f>L1269*G1269</f>
         <v/>
       </c>
     </row>
     <row r="1270">
-      <c r="G1270" s="7" t="n"/>
+      <c r="A1270" s="5" t="inlineStr">
+        <is>
+          <t>Urza, Prince of Kroog / Urza, Príncipe de Kroog</t>
+        </is>
+      </c>
+      <c r="B1270" s="5" t="inlineStr">
+        <is>
+          <t>Legendary Creature — Human Artificer / Criatura Lendária — Humano Artesão</t>
+        </is>
+      </c>
+      <c r="C1270" s="5" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D1270" s="5" t="inlineStr">
+        <is>
+          <t>Artifact creatures you control get +2/+2. {6}: Create a token that's a copy of target artifact you control, except it's a 1/1 Soldier creature in addition to its other types. / As criaturas artefato que você controla recebem +2/+2. {6}: Crie uma ficha que seja uma cópia do artefato alvo que você controla, exceto por ser uma criatura Soldado 1/1 além de seus outros tipos.</t>
+        </is>
+      </c>
+      <c r="E1270" s="5" t="inlineStr">
+        <is>
+          <t>{2}{W}{U}</t>
+        </is>
+      </c>
+      <c r="F1270" s="5" t="inlineStr">
+        <is>
+          <t>Azul, Branco</t>
+        </is>
+      </c>
+      <c r="G1270" s="7" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H1270" s="5" t="inlineStr">
+        <is>
+          <t>The Brothers' War (BRO)</t>
+        </is>
+      </c>
+      <c r="I1270" s="5" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J1270" s="5" t="n">
+        <v>2022</v>
+      </c>
+      <c r="K1270" s="8" t="n">
+        <v>46083</v>
+      </c>
+      <c r="L1270" s="5" t="n">
+        <v>1</v>
+      </c>
       <c r="M1270" s="7">
         <f>L1270*G1270</f>
         <v/>
@@ -77680,12 +78184,12 @@
     <row r="1989">
       <c r="A1989" s="0" t="inlineStr">
         <is>
-          <t>Gyre Engineer / Engenheiro da Espiral</t>
+          <t>Naya Charm / Medalhão de Naya</t>
         </is>
       </c>
       <c r="B1989" s="0" t="inlineStr">
         <is>
-          <t>Creature — Vedalken Wizard / Criatura — Vedalkeano Mago</t>
+          <t>Instant / Mágica Instantânea</t>
         </is>
       </c>
       <c r="C1989" s="0" t="inlineStr">
@@ -77695,23 +78199,23 @@
       </c>
       <c r="D1989" s="0" t="inlineStr">
         <is>
-          <t>{T}: Add {G}{U}. / {T}: Adicione {G}{U}.</t>
+          <t>Choose one — • Naya Charm deals 3 damage to target creature. • Return target card from a graveyard to its owner's hand. • Tap all creatures target player controls. / Escolha um — • Medalhão de Naya causa 3 pontos de dano à criatura alvo. • Devolva o card alvo de um cemitério para a mão de seu dono. • Vire todas as criaturas que o jogador alvo controla.</t>
         </is>
       </c>
       <c r="E1989" s="0" t="inlineStr">
         <is>
-          <t>{1}{G}{U}</t>
+          <t>{R}{G}{W}</t>
         </is>
       </c>
       <c r="F1989" s="0" t="inlineStr">
         <is>
-          <t>Verde, Azul</t>
+          <t>Verde, Vermelho, Branco</t>
         </is>
       </c>
       <c r="G1989" s="0" t="inlineStr"/>
       <c r="H1989" s="0" t="inlineStr">
         <is>
-          <t>Ravnica Allegiance (RNA)</t>
+          <t>Shards of Alara (ALA)</t>
         </is>
       </c>
       <c r="I1989" s="0" t="inlineStr">
@@ -77721,14 +78225,10 @@
       </c>
       <c r="J1989" s="0" t="inlineStr">
         <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="K1989" s="0" t="inlineStr">
-        <is>
-          <t>1/1</t>
-        </is>
-      </c>
+          <t>2008</t>
+        </is>
+      </c>
+      <c r="K1989" s="0" t="inlineStr"/>
       <c r="L1989" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -77738,12 +78238,12 @@
     <row r="1990">
       <c r="A1990" s="0" t="inlineStr">
         <is>
-          <t>Shapers' Sanctuary / Santuário dos Moldadores</t>
+          <t>Mishra, Artificer Prodigy / Mishra, Prodígio Artífice</t>
         </is>
       </c>
       <c r="B1990" s="0" t="inlineStr">
         <is>
-          <t>Enchantment / Encantamento</t>
+          <t>Legendary Creature — Human Artificer / Criatura Lendária — Artesão Humano</t>
         </is>
       </c>
       <c r="C1990" s="0" t="inlineStr">
@@ -77753,23 +78253,23 @@
       </c>
       <c r="D1990" s="0" t="inlineStr">
         <is>
-          <t>Whenever a creature you control becomes the target of a spell or ability an opponent controls, you may draw a card. / Toda vez que uma criatura que você controla se torna alvo de uma mágica ou habilidade que um oponente controla, você pode comprar um card.</t>
+          <t>Whenever you cast an artifact spell, you may search your graveyard, hand, and/or library for a card with the same name as that spell and put it onto the battlefield. If you search your library this way, shuffle. / Toda vez que você joga uma mágica de artefato, você pode procurar em seu cemitério, mão e/ou grimório por um card com o mesmo nome daquela mágica e colocá-lo em jogo. Se procurar em seu grimório desta maneira, embaralhe-o.</t>
         </is>
       </c>
       <c r="E1990" s="0" t="inlineStr">
         <is>
-          <t>{G}</t>
+          <t>{1}{U}{B}{R}</t>
         </is>
       </c>
       <c r="F1990" s="0" t="inlineStr">
         <is>
-          <t>Verde</t>
+          <t>Preto, Vermelho, Azul</t>
         </is>
       </c>
       <c r="G1990" s="0" t="inlineStr"/>
       <c r="H1990" s="0" t="inlineStr">
         <is>
-          <t>Ixalan (XLN)</t>
+          <t>Time Spiral (TSP)</t>
         </is>
       </c>
       <c r="I1990" s="0" t="inlineStr">
@@ -77779,10 +78279,14 @@
       </c>
       <c r="J1990" s="0" t="inlineStr">
         <is>
-          <t>2017</t>
-        </is>
-      </c>
-      <c r="K1990" s="0" t="inlineStr"/>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="K1990" s="0" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
       <c r="L1990" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -77792,38 +78296,38 @@
     <row r="1991">
       <c r="A1991" s="0" t="inlineStr">
         <is>
-          <t>Reknit / Retramar</t>
+          <t>Doran, Besieged by Time</t>
         </is>
       </c>
       <c r="B1991" s="0" t="inlineStr">
         <is>
-          <t>Instant / Mágica Instantânea</t>
+          <t>Legendary Creature — Treefolk Druid</t>
         </is>
       </c>
       <c r="C1991" s="0" t="inlineStr">
         <is>
-          <t>Uncommon / Incomum</t>
+          <t>Rare / Rara</t>
         </is>
       </c>
       <c r="D1991" s="0" t="inlineStr">
         <is>
-          <t>Regenerate target permanent. / Regenere a permanente alvo.</t>
+          <t>Each creature spell you cast with toughness greater than its power costs {1} less to cast. Whenever a creature you control attacks or blocks, it gets +X/+X until end of turn, where X is the difference between its power and toughness.</t>
         </is>
       </c>
       <c r="E1991" s="0" t="inlineStr">
         <is>
-          <t>{1}{G/W}</t>
+          <t>{1}{W}{B}{G}</t>
         </is>
       </c>
       <c r="F1991" s="0" t="inlineStr">
         <is>
-          <t>Verde, Branco</t>
+          <t>Preto, Verde, Branco</t>
         </is>
       </c>
       <c r="G1991" s="0" t="inlineStr"/>
       <c r="H1991" s="0" t="inlineStr">
         <is>
-          <t>Shadowmoor (SHM)</t>
+          <t>Lorwyn Eclipsed (ECL)</t>
         </is>
       </c>
       <c r="I1991" s="0" t="inlineStr">
@@ -77833,10 +78337,14 @@
       </c>
       <c r="J1991" s="0" t="inlineStr">
         <is>
-          <t>2008</t>
-        </is>
-      </c>
-      <c r="K1991" s="0" t="inlineStr"/>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="K1991" s="0" t="inlineStr">
+        <is>
+          <t>0/5</t>
+        </is>
+      </c>
       <c r="L1991" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -77846,12 +78354,12 @@
     <row r="1992">
       <c r="A1992" s="0" t="inlineStr">
         <is>
-          <t>Valeron Outlander / Forasteiro de Valeron</t>
+          <t>Shattering Blow / Golpe Despedaçador</t>
         </is>
       </c>
       <c r="B1992" s="0" t="inlineStr">
         <is>
-          <t>Creature — Human Scout / Criatura — Humano Batedor</t>
+          <t>Instant / Mágica Instantânea</t>
         </is>
       </c>
       <c r="C1992" s="0" t="inlineStr">
@@ -77861,23 +78369,23 @@
       </c>
       <c r="D1992" s="0" t="inlineStr">
         <is>
-          <t>Protection from black / Proteção contra o preto</t>
+          <t>Exile target artifact. / Exile o artefato alvo.</t>
         </is>
       </c>
       <c r="E1992" s="0" t="inlineStr">
         <is>
-          <t>{G}{W}</t>
+          <t>{1}{R/W}</t>
         </is>
       </c>
       <c r="F1992" s="0" t="inlineStr">
         <is>
-          <t>Verde, Branco</t>
+          <t>Vermelho, Branco</t>
         </is>
       </c>
       <c r="G1992" s="0" t="inlineStr"/>
       <c r="H1992" s="0" t="inlineStr">
         <is>
-          <t>Conflux (CON)</t>
+          <t>Gatecrash (GTC)</t>
         </is>
       </c>
       <c r="I1992" s="0" t="inlineStr">
@@ -77887,14 +78395,10 @@
       </c>
       <c r="J1992" s="0" t="inlineStr">
         <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="K1992" s="0" t="inlineStr">
-        <is>
-          <t>2/2</t>
-        </is>
-      </c>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="K1992" s="0" t="inlineStr"/>
       <c r="L1992" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -77904,12 +78408,12 @@
     <row r="1993">
       <c r="A1993" s="0" t="inlineStr">
         <is>
-          <t>Sundering Growth / Crescimento Despedaçador</t>
+          <t>Pursue the Past</t>
         </is>
       </c>
       <c r="B1993" s="0" t="inlineStr">
         <is>
-          <t>Instant / Mágica Instantânea</t>
+          <t>Sorcery</t>
         </is>
       </c>
       <c r="C1993" s="0" t="inlineStr">
@@ -77919,23 +78423,23 @@
       </c>
       <c r="D1993" s="0" t="inlineStr">
         <is>
-          <t>Destroy target artifact or enchantment, then populate. (Create a token that's a copy of a creature token you control.) / Destrua o artefato ou encantamento alvo e depois povoe. (Coloque no campo de batalha uma ficha que seja uma cópia de uma ficha de criatura que você controla.)</t>
+          <t>You gain 2 life. You may discard a card. If you do, draw two cards. Flashback {2}{R}{W} (You may cast this card from your graveyard for its flashback cost. Then exile it.)</t>
         </is>
       </c>
       <c r="E1993" s="0" t="inlineStr">
         <is>
-          <t>{G/W}{G/W}</t>
+          <t>{R}{W}</t>
         </is>
       </c>
       <c r="F1993" s="0" t="inlineStr">
         <is>
-          <t>Verde, Branco</t>
+          <t>Vermelho, Branco</t>
         </is>
       </c>
       <c r="G1993" s="0" t="inlineStr"/>
       <c r="H1993" s="0" t="inlineStr">
         <is>
-          <t>Return to Ravnica (RTR)</t>
+          <t>Secrets of Strixhaven (SOS)</t>
         </is>
       </c>
       <c r="I1993" s="0" t="inlineStr">
@@ -77945,7 +78449,7 @@
       </c>
       <c r="J1993" s="0" t="inlineStr">
         <is>
-          <t>2012</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="K1993" s="0" t="inlineStr"/>
@@ -77958,12 +78462,12 @@
     <row r="1994">
       <c r="A1994" s="0" t="inlineStr">
         <is>
-          <t>Architects of Will / Arquitetos do Arbítrio</t>
+          <t>Senate Griffin / Grifo do Senado</t>
         </is>
       </c>
       <c r="B1994" s="0" t="inlineStr">
         <is>
-          <t>Artifact Creature — Human Wizard / Criatura Artefato — Humano Mago</t>
+          <t>Creature — Griffin / Criatura — Grifo</t>
         </is>
       </c>
       <c r="C1994" s="0" t="inlineStr">
@@ -77973,23 +78477,23 @@
       </c>
       <c r="D1994" s="0" t="inlineStr">
         <is>
-          <t>When this creature enters, look at the top three cards of target player's library, then put them back in any order. Cycling {U/B} ({U/B}, Discard this card: Draw a card.) / Quando Arquitetos do Arbítrio entrar em jogo, olhe os três cards do topo do grimório do jogador alvo, depois coloque-os de volta em qualquer ordem. Reciclar {U/B} ({U/B}, Descarte este card: Compre um card.)</t>
+          <t>Flying When this creature enters, scry 1. / Voar Quando Grifo do Senado entrar no campo de batalha, use vidência 1.</t>
         </is>
       </c>
       <c r="E1994" s="0" t="inlineStr">
         <is>
-          <t>{2}{U}{B}</t>
+          <t>{2}{W/U}{W/U}</t>
         </is>
       </c>
       <c r="F1994" s="0" t="inlineStr">
         <is>
-          <t>Preto, Azul</t>
+          <t>Azul, Branco</t>
         </is>
       </c>
       <c r="G1994" s="0" t="inlineStr"/>
       <c r="H1994" s="0" t="inlineStr">
         <is>
-          <t>Alara Reborn (ARB)</t>
+          <t>Ravnica Allegiance (RNA)</t>
         </is>
       </c>
       <c r="I1994" s="0" t="inlineStr">
@@ -77999,12 +78503,12 @@
       </c>
       <c r="J1994" s="0" t="inlineStr">
         <is>
-          <t>2009</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="K1994" s="0" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>3/2</t>
         </is>
       </c>
       <c r="L1994" s="0" t="inlineStr">
@@ -78016,38 +78520,38 @@
     <row r="1995">
       <c r="A1995" s="0" t="inlineStr">
         <is>
-          <t>Spread the Sickness / Difundir a Doença</t>
+          <t>Tannuk, Memorial Ensign</t>
         </is>
       </c>
       <c r="B1995" s="0" t="inlineStr">
         <is>
-          <t>Sorcery / Feitiço</t>
+          <t>Legendary Creature — Kavu Pilot</t>
         </is>
       </c>
       <c r="C1995" s="0" t="inlineStr">
         <is>
-          <t>Common / Comum</t>
+          <t>Uncommon / Incomum</t>
         </is>
       </c>
       <c r="D1995" s="0" t="inlineStr">
         <is>
-          <t>Destroy target creature, then proliferate. (Choose any number of permanents and/or players, then give each another counter of each kind already there.) / Destrua a criatura alvo e depois prolifere. (Você escolhe um número qualquer de permanentes e/ou jogadores com marcadores sobre eles e depois dá a cada um outro marcador de um tipo que eles já tenham.)</t>
+          <t>Landfall — Whenever a land you control enters, Tannuk deals 1 damage to each opponent. If this is the second time this ability has resolved this turn, draw a card.</t>
         </is>
       </c>
       <c r="E1995" s="0" t="inlineStr">
         <is>
-          <t>{4}{B}</t>
+          <t>{1}{R}{G}</t>
         </is>
       </c>
       <c r="F1995" s="0" t="inlineStr">
         <is>
-          <t>Preto</t>
+          <t>Verde, Vermelho</t>
         </is>
       </c>
       <c r="G1995" s="0" t="inlineStr"/>
       <c r="H1995" s="0" t="inlineStr">
         <is>
-          <t>Mirrodin Besieged (MBS)</t>
+          <t>Edge of Eternities (EOE)</t>
         </is>
       </c>
       <c r="I1995" s="0" t="inlineStr">
@@ -78057,10 +78561,14 @@
       </c>
       <c r="J1995" s="0" t="inlineStr">
         <is>
-          <t>2011</t>
-        </is>
-      </c>
-      <c r="K1995" s="0" t="inlineStr"/>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="K1995" s="0" t="inlineStr">
+        <is>
+          <t>2/4</t>
+        </is>
+      </c>
       <c r="L1995" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -78070,38 +78578,38 @@
     <row r="1996">
       <c r="A1996" s="0" t="inlineStr">
         <is>
-          <t>Fathom Feeder / Alimentador das Profundezas</t>
+          <t>Munitions Expert / Especialista em Municiamento</t>
         </is>
       </c>
       <c r="B1996" s="0" t="inlineStr">
         <is>
-          <t>Creature — Eldrazi Drone / Criatura — Eldrazi Zangão</t>
+          <t>Creature — Goblin / Criatura — Goblin</t>
         </is>
       </c>
       <c r="C1996" s="0" t="inlineStr">
         <is>
-          <t>Rare / Rara</t>
+          <t>Uncommon / Incomum</t>
         </is>
       </c>
       <c r="D1996" s="0" t="inlineStr">
         <is>
-          <t>Devoid (This card has no color.) Deathtouch Ingest (Whenever this creature deals combat damage to a player, that player exiles the top card of their library.) {3}{U}{B}: Draw a card. Each opponent exiles the top card of their library. / Desprovido (Este card não tem cor.)Toque mortíferoIngerir (Toda vez que esta criatura causa dano de combate a um jogador, ele exila o card do topo do próprio grimório.){3}{U}{B}: Compre um card. Cada oponente exila o card do topo do próprio grimório.</t>
+          <t>Flash When this creature enters, you may have it deal damage to target creature or planeswalker equal to the number of Goblins you control. / Lampejo Quando Especialista em Municiamento entra no campo de batalha, você pode fazer com que ele cause à criatura ou ao planeswalker alvo dano igual ao número de Goblins que você controla.</t>
         </is>
       </c>
       <c r="E1996" s="0" t="inlineStr">
         <is>
-          <t>{U}{B}</t>
+          <t>{B}{R}</t>
         </is>
       </c>
       <c r="F1996" s="0" t="inlineStr">
         <is>
-          <t>Preto, Azul</t>
+          <t>Preto, Vermelho</t>
         </is>
       </c>
       <c r="G1996" s="0" t="inlineStr"/>
       <c r="H1996" s="0" t="inlineStr">
         <is>
-          <t>Battle for Zendikar (BFZ)</t>
+          <t>Modern Horizons (MH1)</t>
         </is>
       </c>
       <c r="I1996" s="0" t="inlineStr">
@@ -78111,7 +78619,7 @@
       </c>
       <c r="J1996" s="0" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="K1996" s="0" t="inlineStr">
@@ -78128,12 +78636,12 @@
     <row r="1997">
       <c r="A1997" s="0" t="inlineStr">
         <is>
-          <t>Consuming Tide / Maré Consumidora</t>
+          <t>Theater of Horrors / Teatro de Horrores</t>
         </is>
       </c>
       <c r="B1997" s="0" t="inlineStr">
         <is>
-          <t>Sorcery / Feitiço</t>
+          <t>Enchantment / Encantamento</t>
         </is>
       </c>
       <c r="C1997" s="0" t="inlineStr">
@@ -78143,33 +78651,33 @@
       </c>
       <c r="D1997" s="0" t="inlineStr">
         <is>
-          <t>Each player chooses a nonland permanent they control. Return all nonland permanents not chosen this way to their owners' hands. Then you draw a card for each opponent who has more cards in their hand than you. / Cada jogador escolhe uma permanente não de terreno que ele controla. Devolva para as mãos de seus donos todas as permanentes não de terreno não escolhidas dessa forma. Em seguida, você compra um card para cada oponente com mais cards na própria mão que você.</t>
+          <t>At the beginning of your upkeep, exile the top card of your library. During your turn, if an opponent lost life this turn, you may play lands and cast spells from among cards exiled with this enchantment. {3}{R}: This enchantment deals 1 damage to target opponent or planeswalker. / No início de sua manutenção, exile o card do topo de seu grimório. Durante o seu turno, se um oponente perdeu pontos de vida neste turno, você pode jogar cards exilados com Teatro de Horrores. {3}{R}: Teatro de Horrores causa 1 ponto de dano ao oponente ou planeswalker alvo.</t>
         </is>
       </c>
       <c r="E1997" s="0" t="inlineStr">
         <is>
-          <t>{2}{U}{U}</t>
+          <t>{1}{B}{R}</t>
         </is>
       </c>
       <c r="F1997" s="0" t="inlineStr">
         <is>
-          <t>Azul</t>
+          <t>Preto, Vermelho</t>
         </is>
       </c>
       <c r="G1997" s="0" t="inlineStr"/>
       <c r="H1997" s="0" t="inlineStr">
         <is>
-          <t>Innistrad: Crimson Vow Promos (PVOW)</t>
+          <t>Ravnica Allegiance (RNA)</t>
         </is>
       </c>
       <c r="I1997" s="0" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="J1997" s="0" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="K1997" s="0" t="inlineStr"/>
@@ -78182,12 +78690,12 @@
     <row r="1998">
       <c r="A1998" s="0" t="inlineStr">
         <is>
-          <t>Inkfathom Infiltrator / Infiltrado Braçatinta</t>
+          <t>Fireblade Artist / Artista da Lâmina de Fogo</t>
         </is>
       </c>
       <c r="B1998" s="0" t="inlineStr">
         <is>
-          <t>Creature — Merfolk Rogue / Criatura — Tritão Ladino</t>
+          <t>Creature — Human Shaman / Criatura — Humano Xamã</t>
         </is>
       </c>
       <c r="C1998" s="0" t="inlineStr">
@@ -78197,23 +78705,23 @@
       </c>
       <c r="D1998" s="0" t="inlineStr">
         <is>
-          <t>This creature can't block and can't be blocked. / Infiltrado Braçatinta não pode bloquear e não pode ser bloqueado.</t>
+          <t>Haste At the beginning of your upkeep, you may sacrifice a creature. When you do, this creature deals 2 damage to target opponent or planeswalker. / Ímpeto No início de sua manutenção, você pode sacrificar uma criatura. Quando você o faz, Artista da Lâmina de Fogo causa 2 pontos de dano ao oponente ou planeswalker alvo.</t>
         </is>
       </c>
       <c r="E1998" s="0" t="inlineStr">
         <is>
-          <t>{U/B}{U/B}</t>
+          <t>{B}{R}</t>
         </is>
       </c>
       <c r="F1998" s="0" t="inlineStr">
         <is>
-          <t>Preto, Azul</t>
+          <t>Preto, Vermelho</t>
         </is>
       </c>
       <c r="G1998" s="0" t="inlineStr"/>
       <c r="H1998" s="0" t="inlineStr">
         <is>
-          <t>Shadowmoor (SHM)</t>
+          <t>Ravnica Allegiance (RNA)</t>
         </is>
       </c>
       <c r="I1998" s="0" t="inlineStr">
@@ -78223,12 +78731,12 @@
       </c>
       <c r="J1998" s="0" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="K1998" s="0" t="inlineStr">
         <is>
-          <t>2/1</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="L1998" s="0" t="inlineStr">
@@ -78240,38 +78748,38 @@
     <row r="1999">
       <c r="A1999" s="0" t="inlineStr">
         <is>
-          <t>With Great Power . . .</t>
+          <t>Sigil Blessing / Bênção da insígnia</t>
         </is>
       </c>
       <c r="B1999" s="0" t="inlineStr">
         <is>
-          <t>Enchantment — Aura</t>
+          <t>Instant / Mágica Instantânea</t>
         </is>
       </c>
       <c r="C1999" s="0" t="inlineStr">
         <is>
-          <t>Rare / Rara</t>
+          <t>Common / Comum</t>
         </is>
       </c>
       <c r="D1999" s="0" t="inlineStr">
         <is>
-          <t>Enchant creature you control Enchanted creature gets +2/+2 for each Aura and Equipment attached to it. All damage that would be dealt to you is dealt to enchanted creature instead.</t>
+          <t>Until end of turn, target creature you control gets +3/+3 and other creatures you control get +1/+1. / Até o final do turno, a criatura alvo que você controla recebe +3/+3 e as outras criaturas que você controla recebem +1/+1.</t>
         </is>
       </c>
       <c r="E1999" s="0" t="inlineStr">
         <is>
-          <t>{3}{W}</t>
+          <t>{G}{W}</t>
         </is>
       </c>
       <c r="F1999" s="0" t="inlineStr">
         <is>
-          <t>Branco</t>
+          <t>Verde, Branco</t>
         </is>
       </c>
       <c r="G1999" s="0" t="inlineStr"/>
       <c r="H1999" s="0" t="inlineStr">
         <is>
-          <t>Through the Omenpaths (OM1)</t>
+          <t>Shards of Alara (ALA)</t>
         </is>
       </c>
       <c r="I1999" s="0" t="inlineStr">
@@ -78281,7 +78789,7 @@
       </c>
       <c r="J1999" s="0" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="K1999" s="0" t="inlineStr"/>
@@ -78294,38 +78802,38 @@
     <row r="2000">
       <c r="A2000" s="0" t="inlineStr">
         <is>
-          <t>Ulasht, the Hate Seed / Ulasht, a Semente do Ódio</t>
+          <t>Nature's Chant / Canto da Natureza</t>
         </is>
       </c>
       <c r="B2000" s="0" t="inlineStr">
         <is>
-          <t>Legendary Creature — Hellion Hydra / Criatura Lendária — Avernal Hidra</t>
+          <t>Instant / Mágica Instantânea</t>
         </is>
       </c>
       <c r="C2000" s="0" t="inlineStr">
         <is>
-          <t>Rare / Rara</t>
+          <t>Common / Comum</t>
         </is>
       </c>
       <c r="D2000" s="0" t="inlineStr">
         <is>
-          <t>Ulasht enters with a +1/+1 counter on it for each other red creature you control and a +1/+1 counter on it for each other green creature you control. {1}, Remove a +1/+1 counter from Ulasht: Choose one — • Ulasht deals 1 damage to target creature. • Create a 1/1 green Saproling creature token. / Ulasht, a Semente do Ódio, entra no campo de batalha com um marcador +1/+1 para cada outra criatura vermelha sob seu controle e um marcador +1/+1 para cada outra criatura verde sob seu controle. {1}, remova um marcador +1/+1 de Ulasht: Escolha um — • Ulasht causa 1 ponto de dano à criatura alvo. • Crie uma ficha de criatura Saprófita verde 1/1.</t>
+          <t>Destroy target artifact or enchantment. / Destrua o artefato ou encantamento alvo.</t>
         </is>
       </c>
       <c r="E2000" s="0" t="inlineStr">
         <is>
-          <t>{2}{R}{G}</t>
+          <t>{1}{G/W}</t>
         </is>
       </c>
       <c r="F2000" s="0" t="inlineStr">
         <is>
-          <t>Verde, Vermelho</t>
+          <t>Verde, Branco</t>
         </is>
       </c>
       <c r="G2000" s="0" t="inlineStr"/>
       <c r="H2000" s="0" t="inlineStr">
         <is>
-          <t>Guildpact (GPT)</t>
+          <t>Modern Horizons (MH1)</t>
         </is>
       </c>
       <c r="I2000" s="0" t="inlineStr">
@@ -78335,14 +78843,10 @@
       </c>
       <c r="J2000" s="0" t="inlineStr">
         <is>
-          <t>2006</t>
-        </is>
-      </c>
-      <c r="K2000" s="0" t="inlineStr">
-        <is>
-          <t>0/0</t>
-        </is>
-      </c>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K2000" s="0" t="inlineStr"/>
       <c r="L2000" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -78352,12 +78856,12 @@
     <row r="2001">
       <c r="A2001" s="0" t="inlineStr">
         <is>
-          <t>Gruul Spellbreaker / Quebra-mágicas Gruul</t>
+          <t>Zaffai and the Tempests</t>
         </is>
       </c>
       <c r="B2001" s="0" t="inlineStr">
         <is>
-          <t>Creature — Ogre Warrior / Criatura — Ogro Guerreiro</t>
+          <t>Legendary Creature — Human Bard Sorcerer</t>
         </is>
       </c>
       <c r="C2001" s="0" t="inlineStr">
@@ -78367,23 +78871,23 @@
       </c>
       <c r="D2001" s="0" t="inlineStr">
         <is>
-          <t>Riot (This creature enters with your choice of a +1/+1 counter or haste.) Trample During your turn, you and this creature have hexproof. / Tumulto (Esta criatura entra no campo de batalha com um marcador +1/+1 ou ímpeto, à sua escolha.) Atropelar Enquanto for o seu turno, você e Quebra-mágicas Gruul têm resistência a magia.</t>
+          <t>Once during each of your turns, you may cast an instant or sorcery spell from your hand without paying its mana cost.</t>
         </is>
       </c>
       <c r="E2001" s="0" t="inlineStr">
         <is>
-          <t>{1}{R}{G}</t>
+          <t>{5}{U}{R}</t>
         </is>
       </c>
       <c r="F2001" s="0" t="inlineStr">
         <is>
-          <t>Verde, Vermelho</t>
+          <t>Vermelho, Azul</t>
         </is>
       </c>
       <c r="G2001" s="0" t="inlineStr"/>
       <c r="H2001" s="0" t="inlineStr">
         <is>
-          <t>Ravnica Allegiance (RNA)</t>
+          <t>Secrets of Strixhaven (SOS)</t>
         </is>
       </c>
       <c r="I2001" s="0" t="inlineStr">
@@ -78393,12 +78897,12 @@
       </c>
       <c r="J2001" s="0" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="K2001" s="0" t="inlineStr">
         <is>
-          <t>3/3</t>
+          <t>5/7</t>
         </is>
       </c>
       <c r="L2001" s="0" t="inlineStr">
@@ -78410,12 +78914,12 @@
     <row r="2002">
       <c r="A2002" s="0" t="inlineStr">
         <is>
-          <t>Judge's Familiar / Familiar do Juiz</t>
+          <t>Saheeli, Sublime Artificer / Saheeli, Artífice Sublime</t>
         </is>
       </c>
       <c r="B2002" s="0" t="inlineStr">
         <is>
-          <t>Creature — Bird / Criatura — Ave</t>
+          <t>Legendary Planeswalker — Saheeli / Planeswalker Lendário — Saheeli</t>
         </is>
       </c>
       <c r="C2002" s="0" t="inlineStr">
@@ -78425,23 +78929,23 @@
       </c>
       <c r="D2002" s="0" t="inlineStr">
         <is>
-          <t>Flying Sacrifice this creature: Counter target instant or sorcery spell unless its controller pays {1}. / Voar Sacrifique Familiar do Juiz: Anule a mágica instantânea ou feitiço alvo a menos que seu controlador pague {1}.</t>
+          <t>Whenever you cast a noncreature spell, create a 1/1 colorless Servo artifact creature token. −2: Target artifact you control becomes a copy of another target artifact or creature you control until end of turn, except it's an artifact in addition to its other types. / Toda vez que você conjurar uma mágica que não seja de criatura, crie uma ficha de criatura artefato incolor 1/1 do tipo Servus. −2: O artefato alvo que você controla se torna uma cópia de outro artefato ou criatura alvo que você controla até o final do turno, com a exceção de ser um artefato além de seus outros tipos.</t>
         </is>
       </c>
       <c r="E2002" s="0" t="inlineStr">
         <is>
-          <t>{W/U}</t>
+          <t>{1}{U/R}{U/R}</t>
         </is>
       </c>
       <c r="F2002" s="0" t="inlineStr">
         <is>
-          <t>Azul, Branco</t>
+          <t>Vermelho, Azul</t>
         </is>
       </c>
       <c r="G2002" s="0" t="inlineStr"/>
       <c r="H2002" s="0" t="inlineStr">
         <is>
-          <t>Return to Ravnica (RTR)</t>
+          <t>War of the Spark (WAR)</t>
         </is>
       </c>
       <c r="I2002" s="0" t="inlineStr">
@@ -78451,14 +78955,10 @@
       </c>
       <c r="J2002" s="0" t="inlineStr">
         <is>
-          <t>2012</t>
-        </is>
-      </c>
-      <c r="K2002" s="0" t="inlineStr">
-        <is>
-          <t>1/1</t>
-        </is>
-      </c>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K2002" s="0" t="inlineStr"/>
       <c r="L2002" s="0" t="inlineStr">
         <is>
           <t>1</t>
@@ -78468,38 +78968,38 @@
     <row r="2003">
       <c r="A2003" s="0" t="inlineStr">
         <is>
-          <t>Urza, Prince of Kroog / Urza, Príncipe de Kroog</t>
+          <t>Crackling Drake / Dragonete Fagulhante</t>
         </is>
       </c>
       <c r="B2003" s="0" t="inlineStr">
         <is>
-          <t>Legendary Creature — Human Artificer / Criatura Lendária — Humano Artesão</t>
+          <t>Creature — Drake / Criatura — Dragonete</t>
         </is>
       </c>
       <c r="C2003" s="0" t="inlineStr">
         <is>
-          <t>Rare / Rara</t>
+          <t>Uncommon / Incomum</t>
         </is>
       </c>
       <c r="D2003" s="0" t="inlineStr">
         <is>
-          <t>Artifact creatures you control get +2/+2. {6}: Create a token that's a copy of target artifact you control, except it's a 1/1 Soldier creature in addition to its other types. / As criaturas artefato que você controla recebem +2/+2. {6}: Crie uma ficha que seja uma cópia do artefato alvo que você controla, exceto por ser uma criatura Soldado 1/1 além de seus outros tipos.</t>
+          <t>Flying Crackling Drake's power is equal to the total number of instant and sorcery cards you own in exile and in your graveyard. When this creature enters, draw a card. / Voar O poder de Dragonete Fagulhante é igual ao número de cards de mágica instantânea e feitiço que você possui no exílio e em seu cemitério. Quando Dragonete Fagulhante entrar no campo de batalha, compre um card.</t>
         </is>
       </c>
       <c r="E2003" s="0" t="inlineStr">
         <is>
-          <t>{2}{W}{U}</t>
+          <t>{U}{U}{R}{R}</t>
         </is>
       </c>
       <c r="F2003" s="0" t="inlineStr">
         <is>
-          <t>Azul, Branco</t>
+          <t>Vermelho, Azul</t>
         </is>
       </c>
       <c r="G2003" s="0" t="inlineStr"/>
       <c r="H2003" s="0" t="inlineStr">
         <is>
-          <t>The Brothers' War (BRO)</t>
+          <t>Guilds of Ravnica (GRN)</t>
         </is>
       </c>
       <c r="I2003" s="0" t="inlineStr">
@@ -78509,65 +79009,633 @@
       </c>
       <c r="J2003" s="0" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="K2003" s="0" t="inlineStr">
         <is>
+          <t>*/4</t>
+        </is>
+      </c>
+      <c r="L2003" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" s="0" t="inlineStr">
+        <is>
+          <t>Stormchaser Mage / Mago Caçador de Tempestades</t>
+        </is>
+      </c>
+      <c r="B2004" s="0" t="inlineStr">
+        <is>
+          <t>Creature — Human Wizard / Criatura — Humano Mago</t>
+        </is>
+      </c>
+      <c r="C2004" s="0" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D2004" s="0" t="inlineStr">
+        <is>
+          <t>Flying, haste Prowess (Whenever you cast a noncreature spell, this creature gets +1/+1 until end of turn.) / Voar, ímpeto Destreza (Toda vez que você conjura uma mágica que não seja de criatura, esta criatura recebe +1/+1 até o final do turno.)</t>
+        </is>
+      </c>
+      <c r="E2004" s="0" t="inlineStr">
+        <is>
+          <t>{U}{R}</t>
+        </is>
+      </c>
+      <c r="F2004" s="0" t="inlineStr">
+        <is>
+          <t>Vermelho, Azul</t>
+        </is>
+      </c>
+      <c r="G2004" s="0" t="inlineStr"/>
+      <c r="H2004" s="0" t="inlineStr">
+        <is>
+          <t>Oath of the Gatewatch (OGW)</t>
+        </is>
+      </c>
+      <c r="I2004" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2004" s="0" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="K2004" s="0" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="L2004" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" s="0" t="inlineStr">
+        <is>
+          <t>Aragorn, King of Gondor / Aragorn, Rei de Gondor</t>
+        </is>
+      </c>
+      <c r="B2005" s="0" t="inlineStr">
+        <is>
+          <t>Legendary Creature — Human Noble / Criatura Lendária — Humano Nobre</t>
+        </is>
+      </c>
+      <c r="C2005" s="0" t="inlineStr">
+        <is>
+          <t>Mythic / Mítica</t>
+        </is>
+      </c>
+      <c r="D2005" s="0" t="inlineStr">
+        <is>
+          <t>Vigilance, lifelink When Aragorn enters, you become the monarch. Whenever Aragorn attacks, up to one target creature can't block this turn. If you're the monarch, creatures can't block this turn. / Vigilância, vínculo com a vida Quando Aragorn, Rei de Gondor, entra no campo de batalha, você se torna o monarca. Toda vez que Aragorn atacar, até uma criatura alvo não pode bloquear neste turno. Se você for o monarca, as criaturas não poderão bloquear neste turno.</t>
+        </is>
+      </c>
+      <c r="E2005" s="0" t="inlineStr">
+        <is>
+          <t>{1}{U}{R}{W}</t>
+        </is>
+      </c>
+      <c r="F2005" s="0" t="inlineStr">
+        <is>
+          <t>Vermelho, Azul, Branco</t>
+        </is>
+      </c>
+      <c r="G2005" s="0" t="inlineStr"/>
+      <c r="H2005" s="0" t="inlineStr">
+        <is>
+          <t>Tales of Middle-earth Commander (LTC)</t>
+        </is>
+      </c>
+      <c r="I2005" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2005" s="0" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="K2005" s="0" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="L2005" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" s="0" t="inlineStr">
+        <is>
+          <t>Galadriel, Elven-Queen / Galadriel, Rainha Élfica</t>
+        </is>
+      </c>
+      <c r="B2006" s="0" t="inlineStr">
+        <is>
+          <t>Legendary Creature — Elf Noble / Criatura Lendária — Elfo Nobre</t>
+        </is>
+      </c>
+      <c r="C2006" s="0" t="inlineStr">
+        <is>
+          <t>Mythic / Mítica</t>
+        </is>
+      </c>
+      <c r="D2006" s="0" t="inlineStr">
+        <is>
+          <t>Will of the council — At the beginning of combat on your turn, if another Elf entered the battlefield under your control this turn, starting with you, each player votes for dominion or guidance. If dominion gets more votes, the Ring tempts you, then you put a +1/+1 counter on your Ring-bearer. If guidance gets more votes or the vote is tied, draw a card. / Vontade do conselho — No início do combate no seu turno, se outro Elfo tiver entrado no campo de batalha sob seu controle neste turno, começando por você, cada jogador vota por domínio ou orientação. Se domínio tiver mais votos, o Anel tentará você e, em seguida, você colocará um marcador +1/+1 em seu Guardião do Anel. Se orientação tiver mais votos ou se a votação estiver empatada, compre um card.</t>
+        </is>
+      </c>
+      <c r="E2006" s="0" t="inlineStr">
+        <is>
+          <t>{2}{G}{U}</t>
+        </is>
+      </c>
+      <c r="F2006" s="0" t="inlineStr">
+        <is>
+          <t>Verde, Azul</t>
+        </is>
+      </c>
+      <c r="G2006" s="0" t="inlineStr"/>
+      <c r="H2006" s="0" t="inlineStr">
+        <is>
+          <t>Tales of Middle-earth Commander (LTC)</t>
+        </is>
+      </c>
+      <c r="I2006" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2006" s="0" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="K2006" s="0" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="L2006" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" s="0" t="inlineStr">
+        <is>
+          <t>Biovisionary / Biovisionário</t>
+        </is>
+      </c>
+      <c r="B2007" s="0" t="inlineStr">
+        <is>
+          <t>Creature — Human Wizard / Criatura — Humano Mago</t>
+        </is>
+      </c>
+      <c r="C2007" s="0" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D2007" s="0" t="inlineStr">
+        <is>
+          <t>At the beginning of the end step, if you control four or more creatures named Biovisionary, you win the game. / No início da etapa final, se você controlar quatro ou mais criaturas com o nome Biovisionário, você ganha o jogo.</t>
+        </is>
+      </c>
+      <c r="E2007" s="0" t="inlineStr">
+        <is>
+          <t>{1}{G}{U}</t>
+        </is>
+      </c>
+      <c r="F2007" s="0" t="inlineStr">
+        <is>
+          <t>Verde, Azul</t>
+        </is>
+      </c>
+      <c r="G2007" s="0" t="inlineStr"/>
+      <c r="H2007" s="0" t="inlineStr">
+        <is>
+          <t>Gatecrash (GTC)</t>
+        </is>
+      </c>
+      <c r="I2007" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2007" s="0" t="inlineStr">
+        <is>
+          <t>2013</t>
+        </is>
+      </c>
+      <c r="K2007" s="0" t="inlineStr">
+        <is>
           <t>2/3</t>
         </is>
       </c>
-      <c r="L2003" s="0" t="inlineStr">
+      <c r="L2007" s="0" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="2004">
-      <c r="A2004" t="inlineStr">
-        <is>
-          <t>Naya</t>
-        </is>
-      </c>
-      <c r="B2004" t="inlineStr">
-        <is>
-          <t>Plane — Alara</t>
-        </is>
-      </c>
-      <c r="C2004" t="inlineStr">
+    <row r="2008">
+      <c r="A2008" s="0" t="inlineStr">
+        <is>
+          <t>Sharktocrab / Tubaropolvoguejo</t>
+        </is>
+      </c>
+      <c r="B2008" s="0" t="inlineStr">
+        <is>
+          <t>Creature — Shark Octopus Crab / Criatura — Peixe Polvo Caranguejo</t>
+        </is>
+      </c>
+      <c r="C2008" s="0" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D2008" s="0" t="inlineStr">
+        <is>
+          <t>{2}{G}{U}: Adapt 1. (If this creature has no +1/+1 counters on it, put a +1/+1 counter on it.) Whenever one or more +1/+1 counters are put on this creature, tap target creature an opponent controls. That creature doesn't untap during its controller's next untap step. / {2}{G}: Adaptar 1. (Se esta criatura não tiver marcadores +1/+1, coloque um marcador +1/+1 nela.) Toda vez que um ou mais marcadores +1/+1 forem colocados em Tubaropolvoguejo, vire a criatura alvo que um oponente controla. Aquela criatura não é desvirada durante a próxima etapa de desvirar de seu controlador.</t>
+        </is>
+      </c>
+      <c r="E2008" s="0" t="inlineStr">
+        <is>
+          <t>{2}{G}{U}</t>
+        </is>
+      </c>
+      <c r="F2008" s="0" t="inlineStr">
+        <is>
+          <t>Verde, Azul</t>
+        </is>
+      </c>
+      <c r="G2008" s="0" t="inlineStr"/>
+      <c r="H2008" s="0" t="inlineStr">
+        <is>
+          <t>Ravnica Allegiance (RNA)</t>
+        </is>
+      </c>
+      <c r="I2008" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2008" s="0" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K2008" s="0" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+      <c r="L2008" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" s="0" t="inlineStr">
+        <is>
+          <t>Control Magic / Controlar Mágica</t>
+        </is>
+      </c>
+      <c r="B2009" s="0" t="inlineStr">
+        <is>
+          <t>Enchantment — Aura</t>
+        </is>
+      </c>
+      <c r="C2009" s="0" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D2009" s="0" t="inlineStr">
+        <is>
+          <t>Enchant creature You control enchanted creature.</t>
+        </is>
+      </c>
+      <c r="E2009" s="0" t="inlineStr">
+        <is>
+          <t>{2}{U}{U}</t>
+        </is>
+      </c>
+      <c r="F2009" s="0" t="inlineStr">
+        <is>
+          <t>Azul</t>
+        </is>
+      </c>
+      <c r="G2009" s="0" t="inlineStr"/>
+      <c r="H2009" s="0" t="inlineStr">
+        <is>
+          <t>Limited Edition Alpha (LEA)</t>
+        </is>
+      </c>
+      <c r="I2009" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2009" s="0" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="K2009" s="0" t="inlineStr"/>
+      <c r="L2009" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" s="0" t="inlineStr">
+        <is>
+          <t>Camaraderie / Camaradagem</t>
+        </is>
+      </c>
+      <c r="B2010" s="0" t="inlineStr">
+        <is>
+          <t>Sorcery / Feitiço</t>
+        </is>
+      </c>
+      <c r="C2010" s="0" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D2010" s="0" t="inlineStr">
+        <is>
+          <t>You gain X life and draw X cards, where X is the number of creatures you control. Creatures you control get +1/+1 until end of turn. / Você ganha X pontos de vida e compra X cards, sendo X o número de criaturas que você controla. As criaturas que você controla recebem +1/+1 até o final do turno.</t>
+        </is>
+      </c>
+      <c r="E2010" s="0" t="inlineStr">
+        <is>
+          <t>{4}{G}{W}</t>
+        </is>
+      </c>
+      <c r="F2010" s="0" t="inlineStr">
+        <is>
+          <t>Verde, Branco</t>
+        </is>
+      </c>
+      <c r="G2010" s="0" t="inlineStr"/>
+      <c r="H2010" s="0" t="inlineStr">
+        <is>
+          <t>Guilds of Ravnica (GRN)</t>
+        </is>
+      </c>
+      <c r="I2010" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2010" s="0" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="K2010" s="0" t="inlineStr"/>
+      <c r="L2010" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" s="0" t="inlineStr">
+        <is>
+          <t>Carnival // Carnage / Carnaval // Carnificina</t>
+        </is>
+      </c>
+      <c r="B2011" s="0" t="inlineStr">
+        <is>
+          <t>Instant // Sorcery / Mágica Instantânea</t>
+        </is>
+      </c>
+      <c r="C2011" s="0" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D2011" s="0" t="inlineStr">
+        <is>
+          <t>Carnival: Carnival deals 1 damage to target creature or planeswalker and 1 damage to that permanent's controller. // Carnage: Carnage deals 3 damage to target opponent. That player discards two cards. / Carnaval causa 1 ponto de dano à criatura ou ao planeswalker alvo e 1 ponto de dano ao controlador daquela permanente.</t>
+        </is>
+      </c>
+      <c r="E2011" s="0" t="inlineStr">
+        <is>
+          <t>{B/R} // {2}{B}{R}</t>
+        </is>
+      </c>
+      <c r="F2011" s="0" t="inlineStr">
+        <is>
+          <t>Preto, Vermelho</t>
+        </is>
+      </c>
+      <c r="G2011" s="0" t="inlineStr"/>
+      <c r="H2011" s="0" t="inlineStr">
+        <is>
+          <t>Ravnica Allegiance (RNA)</t>
+        </is>
+      </c>
+      <c r="I2011" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2011" s="0" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="K2011" s="0" t="inlineStr"/>
+      <c r="L2011" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" s="0" t="inlineStr">
+        <is>
+          <t>Psychic Symbiont / Simbionte Psíquico</t>
+        </is>
+      </c>
+      <c r="B2012" s="0" t="inlineStr">
+        <is>
+          <t>Creature — Nightmare Horror / Criatura — Pesadelo Horror</t>
+        </is>
+      </c>
+      <c r="C2012" s="0" t="inlineStr">
+        <is>
+          <t>Uncommon / Incomum</t>
+        </is>
+      </c>
+      <c r="D2012" s="0" t="inlineStr">
+        <is>
+          <t>Flying When this creature enters, target opponent discards a card and you draw a card. / Voar Quando Simbionte Psíquico entra no campo de batalha, o oponente alvo descarta um card e você compra um card.</t>
+        </is>
+      </c>
+      <c r="E2012" s="0" t="inlineStr">
+        <is>
+          <t>{4}{U}{B}</t>
+        </is>
+      </c>
+      <c r="F2012" s="0" t="inlineStr">
+        <is>
+          <t>Preto, Azul</t>
+        </is>
+      </c>
+      <c r="G2012" s="0" t="inlineStr"/>
+      <c r="H2012" s="0" t="inlineStr">
+        <is>
+          <t>Core Set 2019 (M19)</t>
+        </is>
+      </c>
+      <c r="I2012" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2012" s="0" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="K2012" s="0" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="L2012" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" s="0" t="inlineStr">
+        <is>
+          <t>Connive // Concoct / Conivente // Concoctante</t>
+        </is>
+      </c>
+      <c r="B2013" s="0" t="inlineStr">
+        <is>
+          <t>Sorcery // Sorcery / Feitiço</t>
+        </is>
+      </c>
+      <c r="C2013" s="0" t="inlineStr">
+        <is>
+          <t>Rare / Rara</t>
+        </is>
+      </c>
+      <c r="D2013" s="0" t="inlineStr">
+        <is>
+          <t>Connive: Gain control of target creature with power 2 or less. // Concoct: Surveil 3, then return a creature card from your graveyard to the battlefield. / Ganhe o controle da criatura alvo com poder igual ou inferior a 2.</t>
+        </is>
+      </c>
+      <c r="E2013" s="0" t="inlineStr">
+        <is>
+          <t>{2}{U/B}{U/B} // {3}{U}{B}</t>
+        </is>
+      </c>
+      <c r="F2013" s="0" t="inlineStr">
+        <is>
+          <t>Preto, Azul</t>
+        </is>
+      </c>
+      <c r="G2013" s="0" t="inlineStr"/>
+      <c r="H2013" s="0" t="inlineStr">
+        <is>
+          <t>Murders at Karlov Manor Commander (MKC)</t>
+        </is>
+      </c>
+      <c r="I2013" s="0" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2013" s="0" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="K2013" s="0" t="inlineStr"/>
+      <c r="L2013" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>Weird // Goblin</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>Token Creature — Weird // Token Creature — Goblin</t>
+        </is>
+      </c>
+      <c r="C2014" t="inlineStr">
         <is>
           <t>Common / Comum</t>
         </is>
       </c>
-      <c r="D2004" t="inlineStr">
-        <is>
-          <t>You may play any number of lands on each of your turns. Whenever chaos ensues, target red, green, or white creature you control gets +1/+1 until end of turn for each land you control.</t>
-        </is>
-      </c>
-      <c r="E2004" t="inlineStr"/>
-      <c r="F2004" t="inlineStr">
-        <is>
-          <t>Incolor</t>
-        </is>
-      </c>
-      <c r="G2004" t="inlineStr"/>
-      <c r="H2004" t="inlineStr">
-        <is>
-          <t>Planechase Planes (OHOP)</t>
-        </is>
-      </c>
-      <c r="I2004" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="J2004" t="inlineStr">
-        <is>
-          <t>2009</t>
-        </is>
-      </c>
-      <c r="K2004" t="inlineStr"/>
-      <c r="L2004" t="inlineStr">
+      <c r="D2014" t="inlineStr">
+        <is>
+          <t>Weird: Defender, flying</t>
+        </is>
+      </c>
+      <c r="E2014" t="inlineStr"/>
+      <c r="F2014" t="inlineStr">
+        <is>
+          <t>Vermelho, Azul</t>
+        </is>
+      </c>
+      <c r="G2014" t="inlineStr"/>
+      <c r="H2014" t="inlineStr">
+        <is>
+          <t>GRN Guild Kit Tokens (TGK1)</t>
+        </is>
+      </c>
+      <c r="I2014" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="J2014" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="K2014" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="L2014" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>